<commit_message>
thekka site estimate and tinghare baato valuation
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/धारापारि नेवारटोल सिंढी निर्माण/धारापारि नेवारटोल सिंढी निर्माण.xlsx
+++ b/बजेट माग estimate/thekka/धारापारि नेवारटोल सिंढी निर्माण/धारापारि नेवारटोल सिंढी निर्माण.xlsx
@@ -181,35 +181,34 @@
     <t>Providing and laying of hand pack locally available Stone soling with 150 to 200 mm thick stones and packing with smaller stone on prepared surface as per Drawing and Technical Specifications.</t>
   </si>
   <si>
+    <t>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications, PCC Grade M 15, Manual Mixing</t>
+  </si>
+  <si>
+    <t>-13% VAT for water</t>
+  </si>
+  <si>
+    <t>-13% VAT for formwork</t>
+  </si>
+  <si>
+    <t>-masonary wall</t>
+  </si>
+  <si>
+    <t>Random Rubble Masonry, Providing and laying of Stone Masonry Work in the Cement Mortar 1:6 in Foundation complete as per Drawing and Technical Specifications.</t>
+  </si>
+  <si>
+    <t>-13% VAT for stone</t>
+  </si>
+  <si>
     <r>
       <t>-</t>
     </r>
     <r>
       <rPr>
         <sz val="12"/>
-        <color rgb="FFFF0000"/>
         <rFont val="Preeti"/>
       </rPr>
       <t>l;9L</t>
     </r>
-  </si>
-  <si>
-    <t>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications, PCC Grade M 15, Manual Mixing</t>
-  </si>
-  <si>
-    <t>-13% VAT for water</t>
-  </si>
-  <si>
-    <t>-13% VAT for formwork</t>
-  </si>
-  <si>
-    <t>-masonary wall</t>
-  </si>
-  <si>
-    <t>Random Rubble Masonry, Providing and laying of Stone Masonry Work in the Cement Mortar 1:6 in Foundation complete as per Drawing and Technical Specifications.</t>
-  </si>
-  <si>
-    <t>-13% VAT for stone</t>
   </si>
 </sst>
 </file>
@@ -220,7 +219,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,48 +292,14 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <name val="Preeti"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Preeti"/>
     </font>
   </fonts>
   <fills count="2">
@@ -412,160 +377,140 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1155,851 +1100,858 @@
   <dimension ref="A1:K45"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
-    <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.6640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="4"/>
+    <col min="8" max="8" width="5" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" style="4" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.109375" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
     </row>
     <row r="2" spans="1:11" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
-      <c r="K5" s="51"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
     </row>
     <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="46" t="s">
+      <c r="A6" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="47" t="s">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="55" t="s">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="14" t="s">
+      <c r="I8" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="15" t="s">
+      <c r="K8" s="17" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="16">
+      <c r="A9" s="18">
         <v>1</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="17"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="16"/>
-      <c r="B10" s="59" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="36">
+      <c r="A10" s="18"/>
+      <c r="B10" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="20">
         <v>1</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="23">
         <f>10+3+5+6+2+5+3</f>
         <v>34</v>
       </c>
-      <c r="E10" s="36">
+      <c r="E10" s="20">
         <v>3</v>
       </c>
-      <c r="F10" s="36">
+      <c r="F10" s="20">
         <f>0.15+0.1</f>
         <v>0.25</v>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="23">
         <f t="shared" ref="G10" si="0">PRODUCT(C10:F10)</f>
         <v>25.5</v>
       </c>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:11" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="39" t="s">
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="20"/>
+    </row>
+    <row r="11" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
+      <c r="B11" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="40"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="43">
+      <c r="C11" s="26"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="28">
         <f>SUM(G10:G10)</f>
         <v>25.5</v>
       </c>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="45">
+      <c r="I11" s="2">
         <v>748.9</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="28">
         <f>G11*I11</f>
         <v>19096.95</v>
       </c>
-      <c r="K11" s="5"/>
+      <c r="K11" s="27"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="16"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="17"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="20"/>
     </row>
     <row r="13" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
+      <c r="A13" s="18">
         <v>2</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
     </row>
     <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="16"/>
-      <c r="B14" s="59" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="36">
+      <c r="A14" s="18"/>
+      <c r="B14" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="20">
         <v>1</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="23">
         <f>D10</f>
         <v>34</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="20">
         <f>E10+E29</f>
         <v>3.45</v>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="20">
         <v>0.15</v>
       </c>
-      <c r="G14" s="38">
+      <c r="G14" s="23">
         <f t="shared" ref="G14" si="1">PRODUCT(C14:F14)</f>
         <v>17.595000000000002</v>
       </c>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="37"/>
-      <c r="K14" s="17"/>
-    </row>
-    <row r="15" spans="1:11" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="39" t="s">
+      <c r="H14" s="20"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="20"/>
+    </row>
+    <row r="15" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="24"/>
+      <c r="B15" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="40"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="43">
+      <c r="C15" s="26"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="28">
         <f>SUM(G14:G14)</f>
         <v>17.595000000000002</v>
       </c>
-      <c r="H15" s="44" t="s">
+      <c r="H15" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="I15" s="45">
+      <c r="I15" s="2">
         <v>4458.5200000000004</v>
       </c>
-      <c r="J15" s="43">
+      <c r="J15" s="28">
         <f>G15*I15</f>
         <v>78447.659400000019</v>
       </c>
-      <c r="K15" s="5"/>
+      <c r="K15" s="27"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="16"/>
-      <c r="B16" s="32" t="s">
+      <c r="A16" s="18"/>
+      <c r="B16" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="18">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="21">
         <f>0.13*G15*14817.6/5</f>
         <v>6778.6074720000015</v>
       </c>
-      <c r="K16" s="17"/>
+      <c r="K16" s="20"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="16"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
     </row>
     <row r="18" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="16">
+      <c r="A18" s="18">
         <v>3</v>
       </c>
-      <c r="B18" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="17"/>
+      <c r="B18" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="20"/>
     </row>
     <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="16"/>
-      <c r="B19" s="59" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="36">
+      <c r="A19" s="18"/>
+      <c r="B19" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="20">
         <v>1</v>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="23">
         <f>D14</f>
         <v>34</v>
       </c>
-      <c r="E19" s="36">
+      <c r="E19" s="20">
         <f>E14</f>
         <v>3.45</v>
       </c>
-      <c r="F19" s="36">
+      <c r="F19" s="20">
         <v>0.1</v>
       </c>
-      <c r="G19" s="38">
+      <c r="G19" s="23">
         <f t="shared" ref="G19:G20" si="2">PRODUCT(C19:F19)</f>
         <v>11.730000000000002</v>
       </c>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="37"/>
-      <c r="K19" s="17"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="20"/>
     </row>
     <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="16"/>
-      <c r="B20" s="59" t="str">
+      <c r="A20" s="18"/>
+      <c r="B20" s="22" t="str">
         <f>B29</f>
         <v>-masonary wall</v>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="20">
         <f>C29</f>
         <v>1</v>
       </c>
-      <c r="D20" s="38">
+      <c r="D20" s="23">
         <f>D29</f>
         <v>34</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="20">
         <f>E29</f>
         <v>0.45</v>
       </c>
-      <c r="F20" s="36">
+      <c r="F20" s="20">
         <f>0.05</f>
         <v>0.05</v>
       </c>
-      <c r="G20" s="38">
+      <c r="G20" s="23">
         <f t="shared" si="2"/>
         <v>0.76500000000000012</v>
       </c>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="37"/>
-      <c r="K20" s="17"/>
-    </row>
-    <row r="21" spans="1:11" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="39" t="s">
+      <c r="H20" s="20"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="20"/>
+    </row>
+    <row r="21" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="24"/>
+      <c r="B21" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="40"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="43">
+      <c r="C21" s="26"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="28">
         <f>SUM(G19:G20)</f>
         <v>12.495000000000003</v>
       </c>
-      <c r="H21" s="44" t="s">
+      <c r="H21" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="I21" s="45">
+      <c r="I21" s="2">
         <v>11587.52</v>
       </c>
-      <c r="J21" s="43">
+      <c r="J21" s="28">
         <f>G21*I21</f>
         <v>144786.06240000002</v>
       </c>
-      <c r="K21" s="5"/>
+      <c r="K21" s="27"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="16"/>
-      <c r="B22" s="32" t="s">
+      <c r="A22" s="18"/>
+      <c r="B22" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="18">
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="21">
         <f>0.13*G21*53818.03/15</f>
         <v>5827.9544687000016</v>
       </c>
-      <c r="K22" s="17"/>
+      <c r="K22" s="20"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="16"/>
-      <c r="B23" s="32" t="s">
+      <c r="A23" s="18"/>
+      <c r="B23" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="18">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="21">
         <f>0.13*G21*21432.6/15</f>
         <v>2320.9362540000002</v>
       </c>
-      <c r="K23" s="17"/>
+      <c r="K23" s="20"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="16"/>
-      <c r="B24" s="32" t="s">
+      <c r="A24" s="18"/>
+      <c r="B24" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="18">
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="21">
         <f>0.13*G21*(25719.12+13573.98+4286.52)/15</f>
         <v>4719.2370498</v>
       </c>
-      <c r="K24" s="17"/>
+      <c r="K24" s="20"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="16"/>
-      <c r="B25" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="18">
+      <c r="A25" s="18"/>
+      <c r="B25" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="21">
         <f>0.13*G21*620/15</f>
         <v>67.139800000000008</v>
       </c>
-      <c r="K25" s="17"/>
+      <c r="K25" s="20"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="16"/>
-      <c r="B26" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
-      <c r="J26" s="18">
+      <c r="A26" s="18"/>
+      <c r="B26" s="31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="21">
         <f>0.13*G21*6685.1/15</f>
         <v>723.92947900000024</v>
       </c>
-      <c r="K26" s="17"/>
+      <c r="K26" s="20"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" s="16"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="17"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="20"/>
     </row>
     <row r="28" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A28" s="16">
+      <c r="A28" s="18">
         <v>4</v>
       </c>
-      <c r="B28" s="35" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="34"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="17"/>
+      <c r="B28" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="20"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="20"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="16"/>
-      <c r="B29" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="C29" s="36">
+      <c r="A29" s="18"/>
+      <c r="B29" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="20">
         <v>1</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D29" s="23">
         <f>D14</f>
         <v>34</v>
       </c>
-      <c r="E29" s="36">
+      <c r="E29" s="20">
         <v>0.45</v>
       </c>
-      <c r="F29" s="36">
+      <c r="F29" s="20">
         <v>0.75</v>
       </c>
-      <c r="G29" s="38">
+      <c r="G29" s="23">
         <f t="shared" ref="G29" si="3">PRODUCT(C29:F29)</f>
         <v>11.475000000000001</v>
       </c>
-      <c r="H29" s="36"/>
-      <c r="I29" s="36"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="17"/>
-    </row>
-    <row r="30" spans="1:11" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="39" t="s">
+      <c r="H29" s="20"/>
+      <c r="I29" s="20"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="20"/>
+    </row>
+    <row r="30" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="24"/>
+      <c r="B30" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="40"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="43">
+      <c r="C30" s="26"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="28">
         <f>SUM(G29:G29)</f>
         <v>11.475000000000001</v>
       </c>
-      <c r="H30" s="44" t="s">
+      <c r="H30" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="I30" s="45">
+      <c r="I30" s="2">
         <v>9878.43</v>
       </c>
-      <c r="J30" s="43">
+      <c r="J30" s="28">
         <f>G30*I30</f>
         <v>113354.98425000002</v>
       </c>
-      <c r="K30" s="5"/>
+      <c r="K30" s="27"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="16"/>
-      <c r="B31" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="18">
+      <c r="A31" s="18"/>
+      <c r="B31" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="20"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="20"/>
+      <c r="J31" s="21">
         <f>0.13*G30*(14808.78)/5</f>
         <v>4418.1995130000005</v>
       </c>
-      <c r="K31" s="17"/>
+      <c r="K31" s="20"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="16"/>
-      <c r="B32" s="32" t="s">
+      <c r="A32" s="18"/>
+      <c r="B32" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="18">
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="21">
         <f>0.13*G30*5863.95/5</f>
         <v>1749.5094825000001</v>
       </c>
-      <c r="K32" s="17"/>
+      <c r="K32" s="20"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="16"/>
-      <c r="B33" s="32" t="s">
+      <c r="A33" s="18"/>
+      <c r="B33" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="18">
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
+      <c r="I33" s="20"/>
+      <c r="J33" s="21">
         <f>0.13*G30*6604.416/5</f>
         <v>1970.4275136000003</v>
       </c>
-      <c r="K33" s="17"/>
+      <c r="K33" s="20"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="16"/>
-      <c r="B34" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="18">
+      <c r="A34" s="18"/>
+      <c r="B34" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="21">
         <f>0.13*G30*310/5</f>
         <v>92.488500000000016</v>
       </c>
-      <c r="K34" s="17"/>
+      <c r="K34" s="20"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" s="16"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="18"/>
-      <c r="K35" s="17"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+      <c r="I35" s="20"/>
+      <c r="J35" s="21"/>
+      <c r="K35" s="20"/>
     </row>
     <row r="36" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2">
+      <c r="A36" s="24">
         <v>5</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C36" s="26">
         <v>1</v>
       </c>
-      <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="7">
+      <c r="D36" s="1"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="27"/>
+      <c r="G36" s="29">
         <f t="shared" ref="G36" si="4">PRODUCT(C36:F36)</f>
         <v>1</v>
       </c>
-      <c r="H36" s="7" t="s">
+      <c r="H36" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="2">
         <v>500</v>
       </c>
-      <c r="J36" s="7">
+      <c r="J36" s="29">
         <f>G36*I36</f>
         <v>500</v>
       </c>
-      <c r="K36" s="5"/>
+      <c r="K36" s="27"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="18"/>
-      <c r="K37" s="5"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="27"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="21"/>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="35"/>
+      <c r="B38" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C38" s="23"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
-      <c r="J38" s="18">
+      <c r="C38" s="37"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21">
         <f>SUM(J9:J36)</f>
         <v>384854.08558260009</v>
       </c>
-      <c r="K38" s="25"/>
-    </row>
-    <row r="40" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="26"/>
-      <c r="B40" s="27" t="s">
+      <c r="K38" s="39"/>
+    </row>
+    <row r="40" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="40"/>
+      <c r="B40" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="C40" s="52">
+      <c r="C40" s="42">
         <f>J38</f>
         <v>384854.08558260009</v>
       </c>
-      <c r="D40" s="53"/>
-      <c r="E40" s="9">
+      <c r="D40" s="43"/>
+      <c r="E40" s="44">
         <v>100</v>
       </c>
-      <c r="F40" s="26"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="30"/>
-      <c r="K40" s="31"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="45"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="46"/>
+      <c r="J40" s="47"/>
+      <c r="K40" s="48"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="C41" s="56">
+      <c r="C41" s="49">
         <v>100000</v>
       </c>
-      <c r="D41" s="57"/>
-      <c r="E41" s="9"/>
+      <c r="D41" s="50"/>
+      <c r="E41" s="44"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B42" s="27" t="s">
+      <c r="B42" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C42" s="56">
+      <c r="C42" s="49">
         <f>C41-C44-C45</f>
         <v>95000</v>
       </c>
-      <c r="D42" s="57"/>
-      <c r="E42" s="9">
+      <c r="D42" s="50"/>
+      <c r="E42" s="44">
         <f>C42/C40*100</f>
         <v>24.684680131740588</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B43" s="27" t="s">
+      <c r="B43" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C43" s="58">
+      <c r="C43" s="51">
         <f>C40-C42</f>
         <v>289854.08558260009</v>
       </c>
-      <c r="D43" s="58"/>
-      <c r="E43" s="9">
+      <c r="D43" s="51"/>
+      <c r="E43" s="44">
         <f>100-E42</f>
         <v>75.315319868259408</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B44" s="27" t="s">
+      <c r="B44" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="C44" s="52">
+      <c r="C44" s="42">
         <f>C41*0.03</f>
         <v>3000</v>
       </c>
-      <c r="D44" s="53"/>
-      <c r="E44" s="9">
+      <c r="D44" s="43"/>
+      <c r="E44" s="44">
         <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B45" s="27" t="s">
+      <c r="B45" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="C45" s="52">
+      <c r="C45" s="42">
         <f>C41*0.02</f>
         <v>2000</v>
       </c>
-      <c r="D45" s="53"/>
-      <c r="E45" s="9">
+      <c r="D45" s="43"/>
+      <c r="E45" s="44">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="A7:F7"/>
@@ -2008,13 +1960,6 @@
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="C43:D43"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>